<commit_message>
Trim adat to siraman; add full reception day (MC, live music, hotel, coordinator)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wedding_Budget.xlsx
+++ b/Wedding_Budget.xlsx
@@ -734,11 +734,11 @@
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Wedding Option A — Jul 2027</t>
+          <t>Wedding Option A — Aug 2027</t>
         </is>
       </c>
       <c r="C16" s="8">
-        <f>Cashflow!F15</f>
+        <f>Cashflow!F16</f>
         <v/>
       </c>
       <c r="D16" s="9">
@@ -749,11 +749,11 @@
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Wedding Option A — Oct 2027</t>
+          <t>Wedding Option A — Nov 2027</t>
         </is>
       </c>
       <c r="C17" s="8">
-        <f>Cashflow!F18</f>
+        <f>Cashflow!F19</f>
         <v/>
       </c>
       <c r="D17" s="9">
@@ -1256,7 +1256,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Subtle wedding at Rooang Dharmawangsa, full Javanese adat (bride is Javanese). A = intimate/lean · B = comfortable/grand. Figures in Rp mio.</t>
+          <t>Subtle Javanese-adat wedding at Rooang. Pre-wed kept to the siraman; full reception day (MC, music, hotel). A = intimate/lean · B = grander. Rp mio.</t>
         </is>
       </c>
     </row>
@@ -1361,282 +1361,282 @@
     <row r="11">
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Venue — Rooang Dharmawangsa</t>
+          <t>Siraman ceremony</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>A: reception slot (akad at home). B: full akad + reception</t>
+          <t>Setaman flowers, seven-spring water, kendi, dawet, tumpeng, simple gendhing</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Reception catering</t>
-        </is>
-      </c>
-      <c r="C12" s="12">
-        <f>C6*C7</f>
-        <v/>
-      </c>
-      <c r="D12" s="12">
-        <f>D6*D7</f>
-        <v/>
+          <t>Siraman family catering</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Guests × rate / guest</t>
+          <t>Home meal for family on the siraman day</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Siraman &amp; midodareni catering</t>
+          <t>Venue — Rooang Dharmawangsa</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Family meals across the two adat days</t>
+          <t>A: reception (akad at home) · B: full akad + reception</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Siraman ceremony</t>
+          <t>Panggih (temu manten) props</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Setaman flowers, seven-spring water, kendi, dawet, tumpeng</t>
+          <t>Kembar mayang ×2, suruh, egg, kacar-kucur, sindur</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Midodareni</t>
+          <t>Penghulu / KUA (akad)</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Decor + ubarampe (offerings) for the seclusion night</t>
+          <t>Officiant outside office hours</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Panggih props</t>
+          <t>Day-of coordinator (akad + reception)</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Kembar mayang ×2, suruh, egg, kacar-kucur grains &amp; coins, sindur</t>
+          <t>Koordinator hari-H — runs the rundown, cues vendors</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Tarub, janur &amp; tuwuhan</t>
+          <t>MC / host (akad + reception)</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Canopy + plants at the gate marking a wedding house</t>
+          <t>Bilingual host keeping the flow</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Pranatacara + gamelan</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+          <t>Reception catering</t>
+        </is>
+      </c>
+      <c r="C18" s="12">
+        <f>C6*C7</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>D6*D7</f>
+        <v/>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Javanese MC + gamelan (A: recorded · B: live ensemble)</t>
+          <t>Guests × rate / guest</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Wedding rings (both)</t>
-        </is>
-      </c>
-      <c r="C19" s="8">
-        <f>Assumptions!C10</f>
-        <v/>
-      </c>
-      <c r="D19" s="8">
-        <f>Assumptions!C10</f>
-        <v/>
+          <t>Reception decor &amp; floral — Rooang</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Linked from Assumptions</t>
+          <t>Subtle &amp; elegant: stage, entrance, aisle, table florals</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Bride — paes MUA + adat busana</t>
+          <t>Entertainment — live music</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Paes ageng + basahan/kebaya across siraman, akad, panggih, resepsi</t>
+          <t>A: acoustic trio · B: full band</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Groom — adat busana</t>
+          <t>Hotel room — bridal suite (1 night)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Beskap/basahan, blangkon, keris — loafers already bought</t>
+          <t>Wedding-night room for the couple</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Family adat attire</t>
+          <t>Wedding cake &amp; dessert</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Coordinated kebaya/beskap for the parents</t>
+          <t>Cake + sweet corner</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Decoration &amp; floral (pelaminan)</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+          <t>Souvenirs / favours</t>
+        </is>
+      </c>
+      <c r="C23" s="12">
+        <f>C6*C8</f>
+        <v/>
+      </c>
+      <c r="D23" s="12">
+        <f>D6*D8</f>
+        <v/>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Javanese stage + reception styling</t>
+          <t>Guests × rate / guest</t>
         </is>
       </c>
     </row>
@@ -1658,175 +1658,197 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Siraman, midodareni, akad, panggih, resepsi</t>
+          <t>Siraman day + wedding day</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Penghulu / KUA (akad)</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
+          <t>Wedding rings (both)</t>
+        </is>
+      </c>
+      <c r="C25" s="8">
+        <f>Assumptions!C10</f>
+        <v/>
+      </c>
+      <c r="D25" s="8">
+        <f>Assumptions!C10</f>
+        <v/>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Officiant outside office hours</t>
+          <t>Linked from Assumptions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Invitations</t>
+          <t>Bride — paes MUA + adat busana</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>A: digital only. B: digital + printed</t>
+          <t>Paes ageng across siraman, akad, reception</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Souvenirs / favours</t>
-        </is>
-      </c>
-      <c r="C27" s="12">
-        <f>C6*C8</f>
-        <v/>
-      </c>
-      <c r="D27" s="12">
-        <f>D6*D8</f>
-        <v/>
+          <t>Groom — adat busana</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Guests × rate / guest</t>
+          <t>Beskap/basahan, blangkon, keris — loafers already bought</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Wedding cake &amp; dessert</t>
+          <t>Family adat attire</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Cake + sweet corner</t>
+          <t>Coordinated kebaya/beskap for the parents</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Mahar (dowry)</t>
+          <t>Invitations</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Symbolic — set to your intention</t>
+          <t>A: digital · B: digital + printed</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="7" t="inlineStr">
         <is>
+          <t>Mahar (dowry)</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Symbolic — set to your intention</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>Transport &amp; misc</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>Two-day logistics, cars, tips</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="17" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="C31" s="18">
-        <f>SUM(C11:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="18">
-        <f>SUM(D11:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="C32" s="18">
+        <f>SUM(C11:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="18">
+        <f>SUM(D11:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>Sum of the line items above</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="15" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Contingency</t>
         </is>
       </c>
-      <c r="C32" s="12">
-        <f>C31*Assumptions!C12</f>
-        <v/>
-      </c>
-      <c r="D32" s="12">
-        <f>D31*Assumptions!C12</f>
-        <v/>
-      </c>
-      <c r="E32" s="20">
+      <c r="C33" s="12">
+        <f>C32*Assumptions!C12</f>
+        <v/>
+      </c>
+      <c r="D33" s="12">
+        <f>D32*Assumptions!C12</f>
+        <v/>
+      </c>
+      <c r="E33" s="20">
         <f>"Buffer @ "&amp;TEXT(Assumptions!C12,"0%")</f>
         <v/>
       </c>
@@ -1838,11 +1860,11 @@
         </is>
       </c>
       <c r="C40" s="27">
-        <f>C31+C32</f>
+        <f>C32+C33</f>
         <v/>
       </c>
       <c r="D40" s="27">
-        <f>D31+D32</f>
+        <f>D32+D33</f>
         <v/>
       </c>
       <c r="E40" s="28" t="inlineStr">
@@ -2417,11 +2439,11 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>Aug 2027</t>
         </is>
       </c>
       <c r="D6" s="8">
-        <f>Cashflow!F15</f>
+        <f>Cashflow!F16</f>
         <v/>
       </c>
       <c r="E6" s="12">
@@ -2445,11 +2467,11 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>Nov 2027</t>
         </is>
       </c>
       <c r="D7" s="8">
-        <f>Cashflow!F18</f>
+        <f>Cashflow!F19</f>
         <v/>
       </c>
       <c r="E7" s="12">
@@ -2517,7 +2539,7 @@
     <row r="14" ht="32" customHeight="1">
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>Option A — full Javanese adat at an intimate scale — is funded with a cushion by autumn 2027. Option B (the grand adat) is a 2028 project, or needs a bigger monthly saving plus angpau.</t>
+          <t>Option A — siraman + a full reception day at an intimate scale — clears around August 2027 and sits on a cushion by Oct–Nov. Option B (grander, ~100 guests) is a 2028 project, or needs a bigger monthly saving plus angpau.</t>
         </is>
       </c>
     </row>

</xml_diff>